<commit_message>
Verify local AI models, add public demo isolation and deployment checks
</commit_message>
<xml_diff>
--- a/reports/Project_Workbook.xlsx
+++ b/reports/Project_Workbook.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluation" sheetId="1" r:id="R4a6287a6578e4772"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery" sheetId="2" r:id="R380362a58ce744ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluation" sheetId="1" r:id="R1dd8eb9ee2e24daf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery" sheetId="2" r:id="R88aa53f3f27a4453"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -709,10 +709,10 @@
         <x:v>Audio transcription</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>Setup required</x:v>
+        <x:v>Live-tested</x:v>
       </x:c>
       <x:c r="C8" s="7" t="str">
-        <x:v>Install faster-whisper and download model</x:v>
+        <x:v>Whisper tiny transcription passed; model download required</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -720,10 +720,10 @@
         <x:v>Neural embeddings</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>Setup required</x:v>
+        <x:v>Live-tested</x:v>
       </x:c>
       <x:c r="C9" s="7" t="str">
-        <x:v>Install sentence-transformers and model</x:v>
+        <x:v>MiniLM semantic retrieval passed; model download required</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -731,10 +731,10 @@
         <x:v>LLM drafting</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>Setup required</x:v>
+        <x:v>Live-tested</x:v>
       </x:c>
       <x:c r="C10" s="7" t="str">
-        <x:v>Install Ollama and configure model</x:v>
+        <x:v>Qwen Transformers draft passed; Ollama alternative untested</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -742,10 +742,10 @@
         <x:v>Public hosting</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>Not deployed</x:v>
+        <x:v>Account needed</x:v>
       </x:c>
       <x:c r="C11" s="7" t="str">
-        <x:v>Local demo only</x:v>
+        <x:v>Render deployment prepared; no public app URL yet</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
@@ -764,15 +764,27 @@
       <x:c r="B13" s="7"/>
       <x:c r="C13" s="7"/>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="2"/>
-      <x:c r="B14" s="2"/>
-      <x:c r="C14" s="2"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="2"/>
-      <x:c r="B15" s="2"/>
-      <x:c r="C15" s="2"/>
+    <x:row r="14" ht="48" customHeight="1">
+      <x:c r="A14" s="7" t="str">
+        <x:v>API and unit tests</x:v>
+      </x:c>
+      <x:c r="B14" s="7" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C14" s="7" t="str">
+        <x:v>All passed including public demo non-persistence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="48" customHeight="1">
+      <x:c r="A15" s="7" t="str">
+        <x:v>Live model tests</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C15" s="7" t="str">
+        <x:v>3 passed; component smoke tests only</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>